<commit_message>
feat: legacy contact import, reactivation tracking, and customer platform expansion
Add dormant legacy_contact segment with Excel import, Communication Center audiences, auto-reactivation on booking/subscription, welcome-back comms, and admin Legacy Contacts/Reactivated reports. Also ships customer migration toolkit, Customer 360 UI, tier-3 billing fields, DCMS plan addons, staff categories, and complaint supervisor routing.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/fixtures/legacy-migration-sample.xlsx
+++ b/fixtures/legacy-migration-sample.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="57">
   <si>
     <t>CWP Legacy Migration Template v1 — Customers phase (LM-6)</t>
   </si>
@@ -26,6 +26,12 @@
     <t>photo_url optional — customer can also upload from portal</t>
   </si>
   <si>
+    <t>legacy_segment=legacy_contact + status=inactive for old phone-only contacts</t>
+  </si>
+  <si>
+    <t>Use Communication Center audience Legacy Contacts for re-engagement campaigns</t>
+  </si>
+  <si>
     <t>legacy_customer_id*</t>
   </si>
   <si>
@@ -77,6 +83,12 @@
     <t>create_login*</t>
   </si>
   <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>legacy_segment</t>
+  </si>
+  <si>
     <t>LEG-9001</t>
   </si>
   <si>
@@ -125,6 +137,9 @@
     <t>Y</t>
   </si>
   <si>
+    <t>active</t>
+  </si>
+  <si>
     <t>LEG-9002</t>
   </si>
   <si>
@@ -147,6 +162,27 @@
   </si>
   <si>
     <t>legacy9002</t>
+  </si>
+  <si>
+    <t>LEG-CONTACT-9876543210</t>
+  </si>
+  <si>
+    <t>Legacy Contact</t>
+  </si>
+  <si>
+    <t>9876543210</t>
+  </si>
+  <si>
+    <t>Imported from mobile contacts</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>inactive</t>
+  </si>
+  <si>
+    <t>legacy_contact</t>
   </si>
 </sst>
 </file>
@@ -527,7 +563,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -548,6 +584,16 @@
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -558,166 +604,243 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:S4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C2" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D2" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="E2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F2" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G2" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="H2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="I2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="J2" t="s">
+        <v>34</v>
+      </c>
+      <c r="K2" t="s">
+        <v>35</v>
+      </c>
+      <c r="L2" t="s">
+        <v>36</v>
+      </c>
+      <c r="M2" t="s">
+        <v>37</v>
+      </c>
+      <c r="N2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O2" t="s">
+        <v>31</v>
+      </c>
+      <c r="P2" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>40</v>
+      </c>
+      <c r="R2" t="s">
+        <v>41</v>
+      </c>
+      <c r="S2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F3" t="s">
         <v>30</v>
       </c>
-      <c r="K2" t="s">
-        <v>31</v>
-      </c>
-      <c r="L2" t="s">
-        <v>32</v>
-      </c>
-      <c r="M2" t="s">
-        <v>33</v>
-      </c>
-      <c r="N2" t="s">
-        <v>34</v>
-      </c>
-      <c r="O2" t="s">
-        <v>27</v>
-      </c>
-      <c r="P2" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C3" t="s">
-        <v>39</v>
-      </c>
-      <c r="D3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="G3" t="s">
+        <v>31</v>
+      </c>
+      <c r="H3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I3" t="s">
+        <v>46</v>
+      </c>
+      <c r="J3" t="s">
+        <v>31</v>
+      </c>
+      <c r="K3" t="s">
+        <v>47</v>
+      </c>
+      <c r="L3" t="s">
+        <v>31</v>
+      </c>
+      <c r="M3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N3" t="s">
+        <v>48</v>
+      </c>
+      <c r="O3" t="s">
+        <v>31</v>
+      </c>
+      <c r="P3" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q3" t="s">
         <v>40</v>
       </c>
-      <c r="F3" t="s">
-        <v>26</v>
-      </c>
-      <c r="G3" t="s">
-        <v>27</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="R3" t="s">
         <v>41</v>
       </c>
-      <c r="I3" t="s">
-        <v>41</v>
-      </c>
-      <c r="J3" t="s">
-        <v>27</v>
-      </c>
-      <c r="K3" t="s">
-        <v>42</v>
-      </c>
-      <c r="L3" t="s">
-        <v>27</v>
-      </c>
-      <c r="M3" t="s">
-        <v>27</v>
-      </c>
-      <c r="N3" t="s">
-        <v>43</v>
-      </c>
-      <c r="O3" t="s">
-        <v>27</v>
-      </c>
-      <c r="P3" t="s">
-        <v>44</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>36</v>
+      <c r="S3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H4" t="s">
+        <v>46</v>
+      </c>
+      <c r="I4" t="s">
+        <v>46</v>
+      </c>
+      <c r="J4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K4" t="s">
+        <v>31</v>
+      </c>
+      <c r="L4" t="s">
+        <v>31</v>
+      </c>
+      <c r="M4" t="s">
+        <v>31</v>
+      </c>
+      <c r="N4" t="s">
+        <v>53</v>
+      </c>
+      <c r="O4" t="s">
+        <v>31</v>
+      </c>
+      <c r="P4" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>54</v>
+      </c>
+      <c r="R4" t="s">
+        <v>55</v>
+      </c>
+      <c r="S4" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>